<commit_message>
Build Q2767 Kubernetes Windows task
</commit_message>
<xml_diff>
--- a/task/任务规格转化.xlsx
+++ b/task/任务规格转化.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格" sheetId="1" r:id="R42c1cfd5f2b8429c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格" sheetId="1" r:id="R41bfe7aa477b463f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -314,7 +314,7 @@
         <x:v>输入来源</x:v>
       </x:c>
       <x:c r="B5" s="5" t="str">
-        <x:v>研发平台准备的虚构现行Namespace、Pod清单、阶段计划和保留项登记</x:v>
+        <x:v>研发平台准备的虚构Namespace、Pod、阶段标签、过渡等级和保留项资料</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
@@ -330,7 +330,7 @@
         <x:v>原始输入文件</x:v>
       </x:c>
       <x:c r="B7" s="5" t="str">
-        <x:v>input_data/current/namespaces.yaml、input_data/current/workloads.yaml、input_data/rollout/stages.csv、input_data/rollout/retained-items.json及README.md</x:v>
+        <x:v>input_data/current/namespaces.yaml、input_data/current/workloads.yaml、input_data/rollout/stages.csv、input_data/rollout/namespace-policy.csv和input_data/rollout/retained-items.json</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
@@ -338,7 +338,7 @@
         <x:v>目标输出文件</x:v>
       </x:c>
       <x:c r="B8" s="5" t="str">
-        <x:v>output/stages三套清单、output/rendered渲染结果、output/results静态记录、output/tools构建入口及output/RELEASE-NOTES.md</x:v>
+        <x:v>output/stages三套Kustomize目录、output/rendered三份渲染清单、output/results下四份记录与output/RELEASE-NOTES.md</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
@@ -346,31 +346,31 @@
         <x:v>核心操作链</x:v>
       </x:c>
       <x:c r="B9" s="5" t="str">
-        <x:v>现行Pod核对→普通Pod安全改写→阶段标签生成→Kustomize构建→清单差异核对→维护窗口说明</x:v>
+        <x:v>现行对象范围确定→普通Pod安全改写→阶段标签安排→Kustomize渲染→差异与保留项记录→发布说明</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
       <x:c r="A10" s="5" t="str">
-        <x:v>阶段标签</x:v>
+        <x:v>Namespace标签</x:v>
       </x:c>
       <x:c r="B10" s="5" t="str">
-        <x:v>build-shared依次使用privileged、baseline和restricted的enforce标签，warn、audit及版本从stages.csv读取</x:v>
+        <x:v>build-shared的阶段值从stages.csv读取，其他Namespace的过渡等级从namespace-policy.csv读取，六个PodSecurity标签全部保留</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
       <x:c r="A11" s="5" t="str">
-        <x:v>工作负载</x:v>
+        <x:v>Pod规格</x:v>
       </x:c>
       <x:c r="B11" s="5" t="str">
-        <x:v>observe引用现行五个Pod，baseline与restricted引用安全版本，所有阶段Pod身份一致</x:v>
+        <x:v>observe引用现行五个Pod，baseline与restricted引用改写后的Pod，三个阶段的Pod身份相同</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
       <x:c r="A12" s="5" t="str">
-        <x:v>安全字段</x:v>
+        <x:v>安全上下文</x:v>
       </x:c>
       <x:c r="B12" s="5" t="str">
-        <x:v>普通Pod设置runAsNonRoot、RuntimeDefault、禁止提权和drop ALL，test-runner以emptyDir替代hostPath</x:v>
+        <x:v>cache-writer和test-runner使用runAsNonRoot、RuntimeDefault、禁止提权和drop ALL，test-runner以emptyDir替换hostPath</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
@@ -378,47 +378,39 @@
         <x:v>保留项</x:v>
       </x:c>
       <x:c r="B13" s="5" t="str">
-        <x:v>legacy-buildkitRuntimeClass和legacy-vendor命名空间只进入静态登记，不生成AdmissionConfiguration对象</x:v>
+        <x:v>legacy-buildkitRuntimeClass和legacy-vendor命名空间只进入保留记录，不生成AdmissionConfiguration对象</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
       <x:c r="A14" s="5" t="str">
-        <x:v>静态结论</x:v>
+        <x:v>材料边界</x:v>
       </x:c>
       <x:c r="B14" s="5" t="str">
-        <x:v>只检查kubectl kustomize渲染清单，不声称准入生效、Pod重新检查或集群允许或拒绝创建</x:v>
+        <x:v>渲染清单仅表示本地准备情况，API Server的真实准入结果由平台管理员上线后查看</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
       <x:c r="A15" s="5" t="str">
-        <x:v>现场职责</x:v>
+        <x:v>完成条件</x:v>
       </x:c>
       <x:c r="B15" s="5" t="str">
-        <x:v>平台管理员应用所选阶段后确认Namespace标签、Pod替换和集群准入日志</x:v>
+        <x:v>三个Kustomize目录可正常构建，标签与阶段资料一致，普通Pod的安全字段正确，保留项、汇总与发布说明完整</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
       <x:c r="A16" s="5" t="str">
-        <x:v>完成条件</x:v>
+        <x:v>可验证点</x:v>
       </x:c>
       <x:c r="B16" s="5" t="str">
-        <x:v>三阶段Kustomize构建成功，标签与计划一致，普通Pod安全字段正确，保留项和现场事项完整</x:v>
+        <x:v>输入对象集合、阶段集合、Pod复合主键、Namespace标签、Pod安全字段、卷类型、保留项负责人、汇总数量和材料边界</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="15" hidden="0" customHeight="1">
-      <x:c r="A17" s="5" t="str">
-        <x:v>可验证点</x:v>
-      </x:c>
-      <x:c r="B17" s="5" t="str">
-        <x:v>输入集合、阶段集合、对象身份、Namespace标签、Pod安全字段、卷类型、保留项负责人、摘要数量和结论边界</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="15" hidden="0" customHeight="1">
-      <x:c r="A18" s="6" t="str">
+      <x:c r="A17" s="6" t="str">
         <x:v>不适合作为评分点的内容</x:v>
       </x:c>
-      <x:c r="B18" s="6" t="str">
-        <x:v>YAML文件拆分、注释、文档顺序、非root用户编号、CSV行序、JSON键序、临时目录、编辑器选择和说明措辞</x:v>
+      <x:c r="B17" s="6" t="str">
+        <x:v>YAML文件拆分、注释、文档顺序、非root用户编号、CSV行序、JSON键序、编辑器选择和不影响职责的措辞</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Clarify q2767 business input source
</commit_message>
<xml_diff>
--- a/task/任务规格转化.xlsx
+++ b/task/任务规格转化.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格" sheetId="1" r:id="R4ffdff15ade14842"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格" sheetId="1" r:id="Re12bddb9611543a3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -314,7 +314,7 @@
         <x:v>输入来源</x:v>
       </x:c>
       <x:c r="B5" s="5" t="str">
-        <x:v>研发平台准备的虚构Namespace、Pod、维护窗口、影响范围、等待预算、观察时间、回退安排、过渡等级和保留项资料</x:v>
+        <x:v>研发平台发布负责人提供的现行Namespace与Pod清单、维护窗口安排、影响范围、等待预算、观察时间、回退安排、过渡等级和保留项登记</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">

</xml_diff>